<commit_message>
[DEV]: Mapping product in progress
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -1,32 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B484FE4B-1439-45B6-AB81-7670CC974C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F3BC8F-13E6-4191-AAB5-889219DB2776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mapping_products" sheetId="1" r:id="rId1"/>
     <sheet name="instructions_for_use" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="169">
   <si>
     <t>Amora</t>
   </si>
@@ -187,150 +198,9 @@
     <t>Purée</t>
   </si>
   <si>
-    <t>keywords</t>
-  </si>
-  <si>
     <t>product_name</t>
   </si>
   <si>
-    <t>AMORA;DOSETTE</t>
-  </si>
-  <si>
-    <t>AMORA;SQUEEZE</t>
-  </si>
-  <si>
-    <t>AMORA;BOCAL</t>
-  </si>
-  <si>
-    <t>MAILLE;VINAIGRE</t>
-  </si>
-  <si>
-    <t>KNORR;GELEE</t>
-  </si>
-  <si>
-    <t>KNORR;TEXTURE</t>
-  </si>
-  <si>
-    <t>AMORA;SEAU</t>
-  </si>
-  <si>
-    <t>AMORA;SAUCE;SALADE;5L</t>
-  </si>
-  <si>
-    <t>AMORA;SAUCE;SALADE;1L</t>
-  </si>
-  <si>
-    <t>HELLMANN;SEAU</t>
-  </si>
-  <si>
-    <t>HELLMANN;NOUVEAUTE</t>
-  </si>
-  <si>
-    <t>HELLMANN;DOSETTE</t>
-  </si>
-  <si>
-    <t>HELLMANN;SQUEEZE</t>
-  </si>
-  <si>
-    <t>HELLMANN;SANDWICH</t>
-  </si>
-  <si>
-    <t>MAILLE;INSPI;SAUCE;VINAIGRETTE</t>
-  </si>
-  <si>
-    <t>MAILLE;CORNICHON</t>
-  </si>
-  <si>
-    <t>MAIZENA;1KG</t>
-  </si>
-  <si>
-    <t>MAIZENA;700</t>
-  </si>
-  <si>
-    <t>TABASCO;150ML</t>
-  </si>
-  <si>
-    <t>TABASCO;350ML</t>
-  </si>
-  <si>
-    <t>TABASCO;NORMAL</t>
-  </si>
-  <si>
-    <t>TVB;6X1KG</t>
-  </si>
-  <si>
-    <t>TVB;MINI;PANE;PALET;HACHE;EMINCE;VEGETALIEN</t>
-  </si>
-  <si>
-    <t>KNORR;FUMET</t>
-  </si>
-  <si>
-    <t>KNORR;BOUILLON;BIO</t>
-  </si>
-  <si>
-    <t>KNORR;CONCENTRE;LIQUIDE</t>
-  </si>
-  <si>
-    <t>KNORR;JUS;DESHYDRATE</t>
-  </si>
-  <si>
-    <t>KNORR;FOND;DESHYDRATE</t>
-  </si>
-  <si>
-    <t>KNORR;MISE EN PLACE;340</t>
-  </si>
-  <si>
-    <t>KNORR;MISE EN PLACE;700</t>
-  </si>
-  <si>
-    <t>KNORR;COURONNEMENT;LEGUMES</t>
-  </si>
-  <si>
-    <t>KNORR;SAUCE;DESHYDRATE</t>
-  </si>
-  <si>
-    <t>KNORR;BOUILLON;GRANULE</t>
-  </si>
-  <si>
-    <t>KNORR;BASE;TOMATE</t>
-  </si>
-  <si>
-    <t>KNORR;TABOULE</t>
-  </si>
-  <si>
-    <t>KNORR;POTAGE</t>
-  </si>
-  <si>
-    <t>KNORR;ROUX;1KG</t>
-  </si>
-  <si>
-    <t>KNORR;ROUX;10KG</t>
-  </si>
-  <si>
-    <t>KNORR;VIANDOX</t>
-  </si>
-  <si>
-    <t>KNORR;SAUCE;LIQUIDE;GARDE DOR</t>
-  </si>
-  <si>
-    <t>KNORR;AIDE;CULINAIRE</t>
-  </si>
-  <si>
-    <t>KNORR;TERRINE;SOUFFLE;GRATIN</t>
-  </si>
-  <si>
-    <t>KNORR;JUS;LIQUIDE</t>
-  </si>
-  <si>
-    <t>KNORR;SAUCE;CUISINE;MONDE</t>
-  </si>
-  <si>
-    <t>KNORR;PUREE</t>
-  </si>
-  <si>
-    <t>KNORR;SAVEUR;INTENSE</t>
-  </si>
-  <si>
     <t>Ce fichier sert de référentiel de mapping pour remplir product_name</t>
   </si>
   <si>
@@ -433,9 +303,6 @@
     <t>Knorr - Concentrés liquide</t>
   </si>
   <si>
-    <t>Knorr - Gelee</t>
-  </si>
-  <si>
     <t>Knorr - Texture</t>
   </si>
   <si>
@@ -454,18 +321,9 @@
     <t>Knorr - Base tomates</t>
   </si>
   <si>
-    <t>Knorr - Sauces elaborees deshydratees</t>
-  </si>
-  <si>
-    <t>Knorr - Bouillons &amp; bouillons granules</t>
-  </si>
-  <si>
     <t>Knorr - Fonds déshydraté</t>
   </si>
   <si>
-    <t>Knorr - Jus deshydrates</t>
-  </si>
-  <si>
     <t>Hellemann's - Sauce sandwich</t>
   </si>
   <si>
@@ -475,9 +333,6 @@
     <t>Amora - Sauces salades 1L</t>
   </si>
   <si>
-    <t>TVB - Mini pané/palet/haché et emincé végétalien</t>
-  </si>
-  <si>
     <t>Knorr - Taboulé</t>
   </si>
   <si>
@@ -511,10 +366,184 @@
     <t>Knorr - Purée</t>
   </si>
   <si>
-    <t>TABASCO;60ML</t>
-  </si>
-  <si>
     <t>description = Maizena 700G*12 → product_name = Maizena - 700g</t>
+  </si>
+  <si>
+    <t>keywords_brands</t>
+  </si>
+  <si>
+    <t>keywords_others</t>
+  </si>
+  <si>
+    <t>MAILLE</t>
+  </si>
+  <si>
+    <t>MAIZENA</t>
+  </si>
+  <si>
+    <t>TABASCO</t>
+  </si>
+  <si>
+    <t>KNORR</t>
+  </si>
+  <si>
+    <t>HELLMANN'S</t>
+  </si>
+  <si>
+    <t>DOSETTE;10ML</t>
+  </si>
+  <si>
+    <t>SEAU;4K7;5KG</t>
+  </si>
+  <si>
+    <t>SAUCE;SALADE;5L</t>
+  </si>
+  <si>
+    <t>SAUCE;SALADE;1L</t>
+  </si>
+  <si>
+    <t>SEAU</t>
+  </si>
+  <si>
+    <t>NOUVEAUTE</t>
+  </si>
+  <si>
+    <t>DOSETTE</t>
+  </si>
+  <si>
+    <t>VINAIGRE</t>
+  </si>
+  <si>
+    <t>CORNICHON</t>
+  </si>
+  <si>
+    <t>1KG</t>
+  </si>
+  <si>
+    <t>700G</t>
+  </si>
+  <si>
+    <t>150ML</t>
+  </si>
+  <si>
+    <t>350ML</t>
+  </si>
+  <si>
+    <t>NORMAL</t>
+  </si>
+  <si>
+    <t>6X1KG</t>
+  </si>
+  <si>
+    <t>MINI;PANE;PALET;HACHE;EMINCE;VEGETALIEN</t>
+  </si>
+  <si>
+    <t>FUMET</t>
+  </si>
+  <si>
+    <t>BOUILLON;BIO</t>
+  </si>
+  <si>
+    <t>JUS;DESHYDRATE</t>
+  </si>
+  <si>
+    <t>FOND;DESHYDRATE</t>
+  </si>
+  <si>
+    <t>TEXTURE</t>
+  </si>
+  <si>
+    <t>COURONNEMENT;LEGUMES</t>
+  </si>
+  <si>
+    <t>SAVEUR;INTENSE</t>
+  </si>
+  <si>
+    <t>SAUCE;DESHYDRATE</t>
+  </si>
+  <si>
+    <t>BASE;TOMATE</t>
+  </si>
+  <si>
+    <t>TABOULE</t>
+  </si>
+  <si>
+    <t>VIANDOX</t>
+  </si>
+  <si>
+    <t>SAUCE;LIQUIDE;GARDE DOR</t>
+  </si>
+  <si>
+    <t>AIDE;CULINAIRE</t>
+  </si>
+  <si>
+    <t>TERRINE;SOUFFLE;GRATIN</t>
+  </si>
+  <si>
+    <t>JUS;LIQUIDE</t>
+  </si>
+  <si>
+    <t>SAUCE;CUISINE;MONDE</t>
+  </si>
+  <si>
+    <t>PUREE</t>
+  </si>
+  <si>
+    <t>AMORA</t>
+  </si>
+  <si>
+    <t>SQUEEZE;SOUPLE;FLAC;FLACON;FLC;KETCHUP</t>
+  </si>
+  <si>
+    <t>BOCAL;POT;SAVORA;BLC</t>
+  </si>
+  <si>
+    <t>SANDWICH;SANDW</t>
+  </si>
+  <si>
+    <t>SQUEEZE;5L;FLC;SCE</t>
+  </si>
+  <si>
+    <t>POTAGE;SOUPE;VELOUTE;CREME</t>
+  </si>
+  <si>
+    <t>MINI</t>
+  </si>
+  <si>
+    <t>TVB - Mini pané/palet/haché et émincé végétalien</t>
+  </si>
+  <si>
+    <t>Knorr - Jus déshydratés</t>
+  </si>
+  <si>
+    <t>Knorr - Gelée</t>
+  </si>
+  <si>
+    <t>Knorr - Sauces élaborées déshydratées</t>
+  </si>
+  <si>
+    <t>Knorr - Bouillons &amp; bouillons granulés</t>
+  </si>
+  <si>
+    <t>MISE EN PLACE;340;MEP</t>
+  </si>
+  <si>
+    <t>MISE EN PLACE;700;MEP</t>
+  </si>
+  <si>
+    <t>INSPI;SAUCE;VINAIGRETTE;VINAIGRET</t>
+  </si>
+  <si>
+    <t>BOUILLON;GRANULE;DESHYD;DESH:ESSENTIEL;1K</t>
+  </si>
+  <si>
+    <t>CONCENTRE;LIQUIDE;LIQU</t>
+  </si>
+  <si>
+    <t>ROUX;BLANC;1KG</t>
+  </si>
+  <si>
+    <t>ROUX;BLANC;10KG</t>
   </si>
 </sst>
 </file>
@@ -583,12 +612,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -600,7 +632,7 @@
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -616,13 +648,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:D48" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:D48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:E48" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Knorr"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -891,283 +930,341 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="47" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="41.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>103</v>
+        <v>56</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>55</v>
+      <c r="C2" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>61</v>
+      <c r="C3" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>62</v>
+      <c r="C4" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>63</v>
+      <c r="C5" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>56</v>
+      <c r="C6" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>57</v>
+      <c r="C7" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>64</v>
+      <c r="C8" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>65</v>
+      <c r="C9" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>66</v>
+      <c r="C10" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>67</v>
+      <c r="C11" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>68</v>
+      <c r="C12" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>69</v>
+      <c r="C13" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>58</v>
+      <c r="C14" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>70</v>
+      <c r="C15" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>71</v>
+      <c r="C16" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>72</v>
+      <c r="C17" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>161</v>
+      <c r="C18" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>73</v>
+      <c r="C19" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1175,13 +1272,16 @@
         <v>24</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>74</v>
+        <v>114</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1189,13 +1289,16 @@
         <v>25</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>75</v>
+        <v>114</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1203,13 +1306,16 @@
         <v>26</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1217,360 +1323,438 @@
         <v>27</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>77</v>
+        <v>5</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C24" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C25" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C26" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C27" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C28" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C29" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C30" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C31" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C32" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C33" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C34" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C35" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C36" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D37" s="3" t="s">
+      <c r="C37" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D37" s="4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C38" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C39" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C39" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C40" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C40" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C41" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C42" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C42" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C43" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C44" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C44" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C45" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C45" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C46" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C46" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C47" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C47" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C48" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>160</v>
+      <c r="C48" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1593,50 +1777,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>108</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>109</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>110</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>111</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>112</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>113</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[MAPPING]: Add keywords for mapping product
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F3BC8F-13E6-4191-AAB5-889219DB2776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865EDBDE-6EF3-4642-9AB2-9E720999399A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mapping_products" sheetId="1" r:id="rId1"/>
@@ -390,12 +390,6 @@
     <t>HELLMANN'S</t>
   </si>
   <si>
-    <t>DOSETTE;10ML</t>
-  </si>
-  <si>
-    <t>SEAU;4K7;5KG</t>
-  </si>
-  <si>
     <t>SAUCE;SALADE;5L</t>
   </si>
   <si>
@@ -417,9 +411,6 @@
     <t>CORNICHON</t>
   </si>
   <si>
-    <t>1KG</t>
-  </si>
-  <si>
     <t>700G</t>
   </si>
   <si>
@@ -447,21 +438,12 @@
     <t>JUS;DESHYDRATE</t>
   </si>
   <si>
-    <t>FOND;DESHYDRATE</t>
-  </si>
-  <si>
     <t>TEXTURE</t>
   </si>
   <si>
     <t>COURONNEMENT;LEGUMES</t>
   </si>
   <si>
-    <t>SAVEUR;INTENSE</t>
-  </si>
-  <si>
-    <t>SAUCE;DESHYDRATE</t>
-  </si>
-  <si>
     <t>BASE;TOMATE</t>
   </si>
   <si>
@@ -471,9 +453,6 @@
     <t>VIANDOX</t>
   </si>
   <si>
-    <t>SAUCE;LIQUIDE;GARDE DOR</t>
-  </si>
-  <si>
     <t>AIDE;CULINAIRE</t>
   </si>
   <si>
@@ -483,9 +462,6 @@
     <t>JUS;LIQUIDE</t>
   </si>
   <si>
-    <t>SAUCE;CUISINE;MONDE</t>
-  </si>
-  <si>
     <t>PUREE</t>
   </si>
   <si>
@@ -495,18 +471,12 @@
     <t>SQUEEZE;SOUPLE;FLAC;FLACON;FLC;KETCHUP</t>
   </si>
   <si>
-    <t>BOCAL;POT;SAVORA;BLC</t>
-  </si>
-  <si>
     <t>SANDWICH;SANDW</t>
   </si>
   <si>
     <t>SQUEEZE;5L;FLC;SCE</t>
   </si>
   <si>
-    <t>POTAGE;SOUPE;VELOUTE;CREME</t>
-  </si>
-  <si>
     <t>MINI</t>
   </si>
   <si>
@@ -531,12 +501,6 @@
     <t>MISE EN PLACE;700;MEP</t>
   </si>
   <si>
-    <t>INSPI;SAUCE;VINAIGRETTE;VINAIGRET</t>
-  </si>
-  <si>
-    <t>BOUILLON;GRANULE;DESHYD;DESH:ESSENTIEL;1K</t>
-  </si>
-  <si>
     <t>CONCENTRE;LIQUIDE;LIQU</t>
   </si>
   <si>
@@ -544,6 +508,42 @@
   </si>
   <si>
     <t>ROUX;BLANC;10KG</t>
+  </si>
+  <si>
+    <t>POTAGE;SOUPE;VELOUTE;CREME;TOMATE;VEL</t>
+  </si>
+  <si>
+    <t>SAUCE;DESHYDRATE;SCE</t>
+  </si>
+  <si>
+    <t>SAUCE;LIQUIDE;GARDE DOR;SCE</t>
+  </si>
+  <si>
+    <t>SAUCE;CUISINE;MONDE;SCE</t>
+  </si>
+  <si>
+    <t>SEAU;4K7;5KG;SEA</t>
+  </si>
+  <si>
+    <t>DOSETTE;10ML;DISTRIB</t>
+  </si>
+  <si>
+    <t>BOCAL;POT;SAVORA;BCL</t>
+  </si>
+  <si>
+    <t>BOUILLON;GRANULE;DESHYD;DESH:ESSENTIEL;1K;SEA;PATE</t>
+  </si>
+  <si>
+    <t>SAVEUR;INTENSE;ASSAIS;LIQBTL</t>
+  </si>
+  <si>
+    <t>FOND;DESHYDRATE;FD;LIANT;FRD</t>
+  </si>
+  <si>
+    <t>INSPI;SAUCE;VINAIGRETTE;VINAIGRET;VINAIGR</t>
+  </si>
+  <si>
+    <t>1KG;1K;EXPRESS</t>
   </si>
 </sst>
 </file>
@@ -649,13 +649,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:E48" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Knorr"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:E48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="3"/>
@@ -936,7 +930,7 @@
     <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="41.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.5703125" style="1" customWidth="1"/>
     <col min="5" max="5" width="47" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -958,7 +952,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -966,16 +960,16 @@
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -983,16 +977,16 @@
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1000,16 +994,16 @@
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1017,16 +1011,16 @@
         <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1034,16 +1028,16 @@
         <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -1051,16 +1045,16 @@
         <v>12</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1071,13 +1065,13 @@
         <v>116</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1088,13 +1082,13 @@
         <v>116</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1105,13 +1099,13 @@
         <v>116</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1122,13 +1116,13 @@
         <v>116</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -1139,13 +1133,13 @@
         <v>116</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1156,13 +1150,13 @@
         <v>112</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
@@ -1173,13 +1167,13 @@
         <v>112</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -1190,13 +1184,13 @@
         <v>112</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1207,13 +1201,13 @@
         <v>113</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1224,13 +1218,13 @@
         <v>113</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1241,13 +1235,13 @@
         <v>114</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1258,13 +1252,13 @@
         <v>114</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1275,13 +1269,13 @@
         <v>114</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1292,13 +1286,13 @@
         <v>114</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1309,13 +1303,13 @@
         <v>5</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1326,10 +1320,10 @@
         <v>5</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1343,7 +1337,7 @@
         <v>115</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>81</v>
@@ -1360,7 +1354,7 @@
         <v>115</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>86</v>
@@ -1377,7 +1371,7 @@
         <v>115</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>87</v>
@@ -1394,10 +1388,10 @@
         <v>115</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1411,7 +1405,7 @@
         <v>115</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>136</v>
+        <v>166</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>94</v>
@@ -1431,7 +1425,7 @@
         <v>33</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1445,7 +1439,7 @@
         <v>115</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>88</v>
@@ -1462,7 +1456,7 @@
         <v>115</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>89</v>
@@ -1479,7 +1473,7 @@
         <v>115</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>90</v>
@@ -1496,7 +1490,7 @@
         <v>115</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>91</v>
@@ -1513,7 +1507,7 @@
         <v>115</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>92</v>
@@ -1530,13 +1524,13 @@
         <v>115</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -1547,10 +1541,10 @@
         <v>115</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1564,7 +1558,7 @@
         <v>115</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>93</v>
@@ -1581,7 +1575,7 @@
         <v>115</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>98</v>
@@ -1598,7 +1592,7 @@
         <v>115</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>99</v>
@@ -1615,7 +1609,7 @@
         <v>115</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>100</v>
@@ -1632,7 +1626,7 @@
         <v>115</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>101</v>
@@ -1649,7 +1643,7 @@
         <v>115</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>102</v>
@@ -1666,7 +1660,7 @@
         <v>115</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>103</v>
@@ -1683,7 +1677,7 @@
         <v>115</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>104</v>
@@ -1700,7 +1694,7 @@
         <v>115</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>105</v>
@@ -1717,7 +1711,7 @@
         <v>115</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>106</v>
@@ -1734,7 +1728,7 @@
         <v>115</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>107</v>
@@ -1751,7 +1745,7 @@
         <v>115</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>108</v>

</xml_diff>

<commit_message>
[DEV]: Add palier for agreement
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865EDBDE-6EF3-4642-9AB2-9E720999399A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF9821F-0008-4CC3-9F9C-C647ED892C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="172">
   <si>
     <t>Amora</t>
   </si>
@@ -544,12 +544,24 @@
   </si>
   <si>
     <t>1KG;1K;EXPRESS</t>
+  </si>
+  <si>
+    <t>palier_dressing+maizena+TVB_25000-35000_uvc</t>
+  </si>
+  <si>
+    <t>palier_dressing+maizena+TVB_35000-40000_uvc</t>
+  </si>
+  <si>
+    <t>palier_dressing+maizena+TVB_superior-40000_uvc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -593,7 +605,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -608,11 +620,35 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="10">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -648,14 +684,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:E48" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:H48" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -924,18 +963,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="52.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>56</v>
       </c>
@@ -951,552 +992,849 @@
       <c r="E1" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="8" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="F2" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="8" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="F3" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="8" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="F4" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G4" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="H4" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="8" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="F5" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="8" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="F6" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="8" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="F7" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="8" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="F8" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="8" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="F9" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G9" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="H9" s="9">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="8" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="F10" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="H10" s="9">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="8" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="F11" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="H11" s="9">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="8" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="F12" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0.12</v>
+      </c>
+      <c r="H12" s="9">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="8" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="F13" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="G13" s="9">
+        <v>0.45</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="8" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="F14" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="G14" s="9">
+        <v>0.4</v>
+      </c>
+      <c r="H14" s="9">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="8" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="F15" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="G15" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="H15" s="9">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="8" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="F16" s="9">
+        <v>1</v>
+      </c>
+      <c r="G16" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H16" s="9">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="8" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="F17" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G17" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="H17" s="9">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="8" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="F18" s="9">
+        <v>1</v>
+      </c>
+      <c r="G18" s="9">
+        <v>1.05</v>
+      </c>
+      <c r="H18" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="8" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="F19" s="9">
+        <v>0.2</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="7" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="F20" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="G20" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="H20" s="9">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="7" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="F21" s="9">
+        <v>0.3</v>
+      </c>
+      <c r="G21" s="9">
+        <v>0.35</v>
+      </c>
+      <c r="H21" s="9">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="7" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="F22" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G22" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="H22" s="9">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="7" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="F23" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G23" s="9">
+        <v>1.25</v>
+      </c>
+      <c r="H23" s="9">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="10" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="F24" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G24" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="H24" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="10" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="1" t="s">
+      <c r="F25" s="9">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H25" s="9">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="10" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="F26" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G26" s="9">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H26" s="9">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="10" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B28" s="1" t="s">
+      <c r="F27" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="G27" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="H27" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="10" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="F28" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="G28" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="H28" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="10" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="F29" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="G29" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="H29" s="9">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="10" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="F30" s="9">
+        <v>1</v>
+      </c>
+      <c r="G30" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H30" s="9">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B31" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="10" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B32" s="1" t="s">
+      <c r="F31" s="9">
+        <v>1.2</v>
+      </c>
+      <c r="G31" s="9">
+        <v>1.25</v>
+      </c>
+      <c r="H31" s="9">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B32" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="C32" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="10" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B33" s="1" t="s">
+      <c r="F32" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G32" s="9">
+        <v>1.45</v>
+      </c>
+      <c r="H32" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="C33" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="10" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="9">
+        <v>1</v>
+      </c>
+      <c r="G33" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H33" s="9">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -1512,8 +1850,17 @@
       <c r="E34" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F34" s="6">
+        <v>1.05</v>
+      </c>
+      <c r="G34" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H34" s="6">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -1529,8 +1876,17 @@
       <c r="E35" s="3" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F35" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="G35" s="6">
+        <v>1</v>
+      </c>
+      <c r="H35" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -1546,8 +1902,17 @@
       <c r="E36" s="3" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="G36" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="H36" s="6">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -1563,8 +1928,17 @@
       <c r="E37" s="3" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="6">
+        <v>1</v>
+      </c>
+      <c r="G37" s="6">
+        <v>1.05</v>
+      </c>
+      <c r="H37" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -1580,8 +1954,17 @@
       <c r="E38" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="G38" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="H38" s="6">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -1597,8 +1980,17 @@
       <c r="E39" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="G39" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="H39" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -1614,8 +2006,17 @@
       <c r="E40" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="G40" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="H40" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -1631,8 +2032,17 @@
       <c r="E41" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="6">
+        <v>1</v>
+      </c>
+      <c r="G41" s="6">
+        <v>1</v>
+      </c>
+      <c r="H41" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -1648,8 +2058,17 @@
       <c r="E42" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="G42" s="6">
+        <v>0.15</v>
+      </c>
+      <c r="H42" s="6">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -1665,8 +2084,17 @@
       <c r="E43" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="G43" s="6">
+        <v>0.6</v>
+      </c>
+      <c r="H43" s="6">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -1682,8 +2110,17 @@
       <c r="E44" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G44" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="H44" s="6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -1699,8 +2136,17 @@
       <c r="E45" s="3" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G45" s="6">
+        <v>1.45</v>
+      </c>
+      <c r="H45" s="6">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -1716,8 +2162,17 @@
       <c r="E46" s="3" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G46" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="H46" s="6">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -1733,8 +2188,17 @@
       <c r="E47" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="6">
+        <v>0.15</v>
+      </c>
+      <c r="G47" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="H47" s="6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -1749,6 +2213,15 @@
       </c>
       <c r="E48" s="3" t="s">
         <v>108</v>
+      </c>
+      <c r="F48" s="6">
+        <v>1.2</v>
+      </c>
+      <c r="G48" s="6">
+        <v>1.3</v>
+      </c>
+      <c r="H48" s="6">
+        <v>1.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[DEV]: Mapping product modified - Columns added for bearing Knorr
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF9821F-0008-4CC3-9F9C-C647ED892C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17987433-1730-4375-B11D-918E7431F438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="175">
   <si>
     <t>Amora</t>
   </si>
@@ -553,6 +553,15 @@
   </si>
   <si>
     <t>palier_dressing+maizena+TVB_superior-40000_uvc</t>
+  </si>
+  <si>
+    <t>palier_knorr_25000-35000_uvc</t>
+  </si>
+  <si>
+    <t>palier_knorr_35000-40000_uvc</t>
+  </si>
+  <si>
+    <t>palier_knorr_superior-40000_uvc</t>
   </si>
 </sst>
 </file>
@@ -605,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -623,23 +632,20 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="13">
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -684,17 +690,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:H48" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:K48" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{5275C952-1BE3-4F8C-914D-044138271CA5}" name="palier_knorr_25000-35000_uvc" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{DEC7AB06-4B54-4173-A4F4-A7451A605C99}" name="palier_knorr_35000-40000_uvc" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{A2C17C36-21F5-4862-AD48-4801B244CECB}" name="palier_knorr_superior-40000_uvc" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -963,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -973,10 +982,12 @@
     <col min="5" max="5" width="46.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="10" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="52.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>56</v>
       </c>
@@ -1001,840 +1012,935 @@
       <c r="H1" s="2" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="I1" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="6">
         <v>0.2</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="6">
         <v>0.3</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="6">
         <v>0.3</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="6">
         <v>0.4</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="6">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="6">
         <v>1.2</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="6">
         <v>1.3</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="6">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="6">
         <v>0.6</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="6">
         <v>0.7</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="6">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="6">
         <v>0.2</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="6">
         <v>0.3</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="6">
         <v>0.1</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="6">
         <v>0.15</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="6">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="6">
         <v>0.3</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="6">
         <v>0.4</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="6">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="6">
         <v>0.2</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="6">
         <v>0.3</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="6">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="6">
         <v>0.3</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="6">
         <v>0.4</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="6">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="6">
         <v>0.1</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="6">
         <v>0.2</v>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="6">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="6">
         <v>0.1</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="6">
         <v>0.12</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="6">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="6">
         <v>0.4</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="6">
         <v>0.45</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="6">
         <v>0.3</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="6">
         <v>0.4</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="6">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="6">
         <v>0.05</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="6">
         <v>0.1</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="6">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="6">
         <v>1</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="6">
         <v>1.1499999999999999</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="6">
         <v>0.2</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="6">
         <v>0.3</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="6">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="6">
         <v>1</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="6">
         <v>1.05</v>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="6">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="6">
         <v>0.2</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="6">
         <v>0.3</v>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="6">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="6">
         <v>0.5</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="6">
         <v>0.6</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="6">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="6">
         <v>0.3</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="6">
         <v>0.35</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="6">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="6">
         <v>2.2000000000000002</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="6">
         <v>2.2000000000000002</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="6">
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="6">
         <v>1.2</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="6">
         <v>1.25</v>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="6">
         <v>1.3</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F24" s="9">
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6">
         <v>1.2</v>
       </c>
-      <c r="G24" s="9">
+      <c r="J24" s="6">
         <v>1.3</v>
       </c>
-      <c r="H24" s="9">
+      <c r="K24" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F25" s="9">
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6">
         <v>1</v>
       </c>
-      <c r="G25" s="9">
+      <c r="J25" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H25" s="9">
+      <c r="K25" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F26" s="9">
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G26" s="9">
+      <c r="J26" s="6">
         <v>1.1499999999999999</v>
       </c>
-      <c r="H26" s="9">
+      <c r="K26" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F27" s="9">
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6">
         <v>1.3</v>
       </c>
-      <c r="G27" s="9">
+      <c r="J27" s="6">
         <v>1.4</v>
       </c>
-      <c r="H27" s="9">
+      <c r="K27" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F28" s="9">
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6">
         <v>1.3</v>
       </c>
-      <c r="G28" s="9">
+      <c r="J28" s="6">
         <v>1.4</v>
       </c>
-      <c r="H28" s="9">
+      <c r="K28" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="F29" s="9">
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6">
         <v>1.3</v>
       </c>
-      <c r="G29" s="9">
+      <c r="J29" s="6">
         <v>1.3</v>
       </c>
-      <c r="H29" s="9">
+      <c r="K29" s="6">
         <v>1.3</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="9">
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6">
         <v>1</v>
       </c>
-      <c r="G30" s="9">
+      <c r="J30" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H30" s="9">
+      <c r="K30" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F31" s="9">
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6">
         <v>1.2</v>
       </c>
-      <c r="G31" s="9">
+      <c r="J31" s="6">
         <v>1.25</v>
       </c>
-      <c r="H31" s="9">
+      <c r="K31" s="6">
         <v>1.3</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F32" s="9">
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6">
         <v>1.4</v>
       </c>
-      <c r="G32" s="9">
+      <c r="J32" s="6">
         <v>1.45</v>
       </c>
-      <c r="H32" s="9">
+      <c r="K32" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F33" s="9">
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6">
         <v>1</v>
       </c>
-      <c r="G33" s="9">
+      <c r="J33" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H33" s="9">
+      <c r="K33" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -1850,17 +1956,19 @@
       <c r="E34" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F34" s="6">
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6">
         <v>1.05</v>
       </c>
-      <c r="G34" s="6">
+      <c r="J34" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H34" s="6">
+      <c r="K34" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -1876,17 +1984,19 @@
       <c r="E35" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="F35" s="6">
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6">
         <v>0.9</v>
       </c>
-      <c r="G35" s="6">
+      <c r="J35" s="6">
         <v>1</v>
       </c>
-      <c r="H35" s="6">
+      <c r="K35" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -1902,17 +2012,19 @@
       <c r="E36" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F36" s="6">
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6">
         <v>1.5</v>
       </c>
-      <c r="G36" s="6">
+      <c r="J36" s="6">
         <v>1.5</v>
       </c>
-      <c r="H36" s="6">
+      <c r="K36" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -1928,17 +2040,19 @@
       <c r="E37" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F37" s="6">
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6">
         <v>1</v>
       </c>
-      <c r="G37" s="6">
+      <c r="J37" s="6">
         <v>1.05</v>
       </c>
-      <c r="H37" s="6">
+      <c r="K37" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -1954,17 +2068,19 @@
       <c r="E38" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F38" s="6">
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6">
         <v>0.8</v>
       </c>
-      <c r="G38" s="6">
+      <c r="J38" s="6">
         <v>0.9</v>
       </c>
-      <c r="H38" s="6">
+      <c r="K38" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -1980,17 +2096,19 @@
       <c r="E39" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F39" s="6">
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6">
         <v>0.6</v>
       </c>
-      <c r="G39" s="6">
+      <c r="J39" s="6">
         <v>0.8</v>
       </c>
-      <c r="H39" s="6">
+      <c r="K39" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -2006,17 +2124,19 @@
       <c r="E40" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F40" s="6">
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6">
         <v>0.9</v>
       </c>
-      <c r="G40" s="6">
+      <c r="J40" s="6">
         <v>0.95</v>
       </c>
-      <c r="H40" s="6">
+      <c r="K40" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -2032,17 +2152,19 @@
       <c r="E41" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F41" s="6">
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6">
         <v>1</v>
       </c>
-      <c r="G41" s="6">
+      <c r="J41" s="6">
         <v>1</v>
       </c>
-      <c r="H41" s="6">
+      <c r="K41" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -2058,17 +2180,19 @@
       <c r="E42" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="F42" s="6">
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6">
         <v>0.1</v>
       </c>
-      <c r="G42" s="6">
+      <c r="J42" s="6">
         <v>0.15</v>
       </c>
-      <c r="H42" s="6">
+      <c r="K42" s="6">
         <v>0.2</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -2084,17 +2208,19 @@
       <c r="E43" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F43" s="6">
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6">
         <v>0.5</v>
       </c>
-      <c r="G43" s="6">
+      <c r="J43" s="6">
         <v>0.6</v>
       </c>
-      <c r="H43" s="6">
+      <c r="K43" s="6">
         <v>0.8</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -2110,17 +2236,19 @@
       <c r="E44" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F44" s="6">
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6">
         <v>0.2</v>
       </c>
-      <c r="G44" s="6">
+      <c r="J44" s="6">
         <v>0.25</v>
       </c>
-      <c r="H44" s="6">
+      <c r="K44" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -2136,17 +2264,19 @@
       <c r="E45" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="6">
+      <c r="G45" s="6"/>
+      <c r="H45" s="6"/>
+      <c r="I45" s="6">
         <v>1.4</v>
       </c>
-      <c r="G45" s="6">
+      <c r="J45" s="6">
         <v>1.45</v>
       </c>
-      <c r="H45" s="6">
+      <c r="K45" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -2162,17 +2292,19 @@
       <c r="E46" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="F46" s="6">
+      <c r="G46" s="6"/>
+      <c r="H46" s="6"/>
+      <c r="I46" s="6">
         <v>0.2</v>
       </c>
-      <c r="G46" s="6">
+      <c r="J46" s="6">
         <v>0.3</v>
       </c>
-      <c r="H46" s="6">
+      <c r="K46" s="6">
         <v>0.4</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2188,17 +2320,19 @@
       <c r="E47" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F47" s="6">
+      <c r="G47" s="6"/>
+      <c r="H47" s="6"/>
+      <c r="I47" s="6">
         <v>0.15</v>
       </c>
-      <c r="G47" s="6">
+      <c r="J47" s="6">
         <v>0.2</v>
       </c>
-      <c r="H47" s="6">
+      <c r="K47" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -2214,13 +2348,15 @@
       <c r="E48" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F48" s="6">
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6">
         <v>1.2</v>
       </c>
-      <c r="G48" s="6">
+      <c r="J48" s="6">
         <v>1.3</v>
       </c>
-      <c r="H48" s="6">
+      <c r="K48" s="6">
         <v>1.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[DEV]: For importation transaction, add possibility choose file mapping_product; for important agreement, add new column for the calculation of income
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17987433-1730-4375-B11D-918E7431F438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D35256-91CB-4186-A958-BB94AFB6EAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="176">
   <si>
     <t>Amora</t>
   </si>
@@ -562,6 +562,9 @@
   </si>
   <si>
     <t>palier_knorr_superior-40000_uvc</t>
+  </si>
+  <si>
+    <t>is_billed_per_case</t>
   </si>
 </sst>
 </file>
@@ -636,7 +639,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -690,20 +696,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:K48" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{5275C952-1BE3-4F8C-914D-044138271CA5}" name="palier_knorr_25000-35000_uvc" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{DEC7AB06-4B54-4173-A4F4-A7451A605C99}" name="palier_knorr_35000-40000_uvc" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{A2C17C36-21F5-4862-AD48-4801B244CECB}" name="palier_knorr_superior-40000_uvc" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:L48" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:L48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{D6F1DC80-59FF-426F-9473-675A434B4902}" name="is_billed_per_case" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{5275C952-1BE3-4F8C-914D-044138271CA5}" name="palier_knorr_25000-35000_uvc" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{DEC7AB06-4B54-4173-A4F4-A7451A605C99}" name="palier_knorr_35000-40000_uvc" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{A2C17C36-21F5-4862-AD48-4801B244CECB}" name="palier_knorr_superior-40000_uvc" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -972,22 +979,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="53.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="52.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="6" width="46.42578125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="52.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>56</v>
       </c>
@@ -1004,25 +1011,28 @@
         <v>53</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1038,20 +1048,23 @@
       <c r="E2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6">
         <v>0.2</v>
       </c>
-      <c r="G2" s="6">
+      <c r="H2" s="6">
         <v>0.3</v>
       </c>
-      <c r="H2" s="6">
+      <c r="I2" s="6">
         <v>0.5</v>
       </c>
-      <c r="I2" s="6"/>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="6"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1067,20 +1080,23 @@
       <c r="E3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="6">
         <v>0.3</v>
       </c>
-      <c r="G3" s="6">
+      <c r="H3" s="6">
         <v>0.4</v>
       </c>
-      <c r="H3" s="6">
+      <c r="I3" s="6">
         <v>0.6</v>
       </c>
-      <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1096,20 +1112,23 @@
       <c r="E4" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="6">
         <v>1.2</v>
       </c>
-      <c r="G4" s="6">
+      <c r="H4" s="6">
         <v>1.3</v>
       </c>
-      <c r="H4" s="6">
+      <c r="I4" s="6">
         <v>1.5</v>
       </c>
-      <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="6"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1125,20 +1144,23 @@
       <c r="E5" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6">
         <v>0.6</v>
       </c>
-      <c r="G5" s="6">
+      <c r="H5" s="6">
         <v>0.7</v>
       </c>
-      <c r="H5" s="6">
+      <c r="I5" s="6">
         <v>0.9</v>
       </c>
-      <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="6"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1154,20 +1176,23 @@
       <c r="E6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
         <v>0.2</v>
       </c>
-      <c r="G6" s="6">
+      <c r="H6" s="6">
         <v>0.3</v>
       </c>
-      <c r="H6" s="6">
+      <c r="I6" s="6">
         <v>0.5</v>
       </c>
-      <c r="I6" s="6"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -1183,20 +1208,23 @@
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6">
         <v>0.1</v>
       </c>
-      <c r="G7" s="6">
+      <c r="H7" s="6">
         <v>0.15</v>
       </c>
-      <c r="H7" s="6">
+      <c r="I7" s="6">
         <v>0.2</v>
       </c>
-      <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1212,20 +1240,23 @@
       <c r="E8" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6">
         <v>0.3</v>
       </c>
-      <c r="G8" s="6">
+      <c r="H8" s="6">
         <v>0.4</v>
       </c>
-      <c r="H8" s="6">
+      <c r="I8" s="6">
         <v>0.6</v>
       </c>
-      <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="6"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1241,20 +1272,23 @@
       <c r="E9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
         <v>0.2</v>
       </c>
-      <c r="G9" s="6">
+      <c r="H9" s="6">
         <v>0.3</v>
       </c>
-      <c r="H9" s="6">
+      <c r="I9" s="6">
         <v>0.4</v>
       </c>
-      <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="6"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1270,20 +1304,23 @@
       <c r="E10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6">
         <v>0.3</v>
       </c>
-      <c r="G10" s="6">
+      <c r="H10" s="6">
         <v>0.4</v>
       </c>
-      <c r="H10" s="6">
+      <c r="I10" s="6">
         <v>0.6</v>
       </c>
-      <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="6"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1299,20 +1336,23 @@
       <c r="E11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6">
         <v>0.1</v>
       </c>
-      <c r="G11" s="6">
+      <c r="H11" s="6">
         <v>0.2</v>
       </c>
-      <c r="H11" s="6">
+      <c r="I11" s="6">
         <v>0.3</v>
       </c>
-      <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="6"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -1328,20 +1368,23 @@
       <c r="E12" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6">
         <v>0.1</v>
       </c>
-      <c r="G12" s="6">
+      <c r="H12" s="6">
         <v>0.12</v>
       </c>
-      <c r="H12" s="6">
+      <c r="I12" s="6">
         <v>0.15</v>
       </c>
-      <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" s="6"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1357,20 +1400,23 @@
       <c r="E13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6">
         <v>0.4</v>
       </c>
-      <c r="G13" s="6">
+      <c r="H13" s="6">
         <v>0.45</v>
       </c>
-      <c r="H13" s="6">
+      <c r="I13" s="6">
         <v>0.5</v>
       </c>
-      <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="6"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
@@ -1386,20 +1432,23 @@
       <c r="E14" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
         <v>0.3</v>
       </c>
-      <c r="G14" s="6">
+      <c r="H14" s="6">
         <v>0.4</v>
       </c>
-      <c r="H14" s="6">
+      <c r="I14" s="6">
         <v>0.45</v>
       </c>
-      <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="6"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -1415,20 +1464,23 @@
       <c r="E15" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6">
         <v>0.05</v>
       </c>
-      <c r="G15" s="6">
+      <c r="H15" s="6">
         <v>0.1</v>
       </c>
-      <c r="H15" s="6">
+      <c r="I15" s="6">
         <v>0.15</v>
       </c>
-      <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="6"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1444,20 +1496,23 @@
       <c r="E16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6">
         <v>1</v>
       </c>
-      <c r="G16" s="6">
+      <c r="H16" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H16" s="6">
+      <c r="I16" s="6">
         <v>1.1499999999999999</v>
       </c>
-      <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16" s="6"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1473,20 +1528,23 @@
       <c r="E17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="G17" s="6">
         <v>0.2</v>
       </c>
-      <c r="G17" s="6">
+      <c r="H17" s="6">
         <v>0.3</v>
       </c>
-      <c r="H17" s="6">
+      <c r="I17" s="6">
         <v>0.5</v>
       </c>
-      <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="6"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1502,20 +1560,23 @@
       <c r="E18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
         <v>1</v>
       </c>
-      <c r="G18" s="6">
+      <c r="H18" s="6">
         <v>1.05</v>
       </c>
-      <c r="H18" s="6">
+      <c r="I18" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" s="6"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1531,20 +1592,23 @@
       <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6">
         <v>0.2</v>
       </c>
-      <c r="G19" s="6">
+      <c r="H19" s="6">
         <v>0.3</v>
       </c>
-      <c r="H19" s="6">
+      <c r="I19" s="6">
         <v>0.4</v>
       </c>
-      <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L19" s="6"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1560,20 +1624,23 @@
       <c r="E20" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6">
         <v>0.5</v>
       </c>
-      <c r="G20" s="6">
+      <c r="H20" s="6">
         <v>0.6</v>
       </c>
-      <c r="H20" s="6">
+      <c r="I20" s="6">
         <v>0.8</v>
       </c>
-      <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="6"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1589,20 +1656,23 @@
       <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="4">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6">
         <v>0.3</v>
       </c>
-      <c r="G21" s="6">
+      <c r="H21" s="6">
         <v>0.35</v>
       </c>
-      <c r="H21" s="6">
+      <c r="I21" s="6">
         <v>0.45</v>
       </c>
-      <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="6"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1618,8 +1688,8 @@
       <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="6">
-        <v>2.2000000000000002</v>
+      <c r="F22" s="4">
+        <v>0</v>
       </c>
       <c r="G22" s="6">
         <v>2.2000000000000002</v>
@@ -1627,11 +1697,14 @@
       <c r="H22" s="6">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I22" s="6"/>
+      <c r="I22" s="6">
+        <v>2.2000000000000002</v>
+      </c>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L22" s="6"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1647,20 +1720,23 @@
       <c r="E23" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="6">
         <v>1.2</v>
       </c>
-      <c r="G23" s="6">
+      <c r="H23" s="6">
         <v>1.25</v>
       </c>
-      <c r="H23" s="6">
+      <c r="I23" s="6">
         <v>1.3</v>
       </c>
-      <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="6"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -1676,19 +1752,22 @@
       <c r="E24" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G24" s="6"/>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
       <c r="H24" s="6"/>
-      <c r="I24" s="6">
+      <c r="I24" s="6"/>
+      <c r="J24" s="6">
         <v>1.2</v>
       </c>
-      <c r="J24" s="6">
+      <c r="K24" s="6">
         <v>1.3</v>
       </c>
-      <c r="K24" s="6">
+      <c r="L24" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -1704,19 +1783,22 @@
       <c r="E25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G25" s="6"/>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
       <c r="H25" s="6"/>
-      <c r="I25" s="6">
+      <c r="I25" s="6"/>
+      <c r="J25" s="6">
         <v>1</v>
       </c>
-      <c r="J25" s="6">
+      <c r="K25" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K25" s="6">
+      <c r="L25" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -1732,19 +1814,22 @@
       <c r="E26" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G26" s="6"/>
+      <c r="F26" s="4">
+        <v>0</v>
+      </c>
       <c r="H26" s="6"/>
-      <c r="I26" s="6">
+      <c r="I26" s="6"/>
+      <c r="J26" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J26" s="6">
+      <c r="K26" s="6">
         <v>1.1499999999999999</v>
       </c>
-      <c r="K26" s="6">
+      <c r="L26" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -1760,19 +1845,22 @@
       <c r="E27" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="G27" s="6"/>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
       <c r="H27" s="6"/>
-      <c r="I27" s="6">
+      <c r="I27" s="6"/>
+      <c r="J27" s="6">
         <v>1.3</v>
       </c>
-      <c r="J27" s="6">
+      <c r="K27" s="6">
         <v>1.4</v>
       </c>
-      <c r="K27" s="6">
+      <c r="L27" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -1788,19 +1876,22 @@
       <c r="E28" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G28" s="6"/>
+      <c r="F28" s="4">
+        <v>0</v>
+      </c>
       <c r="H28" s="6"/>
-      <c r="I28" s="6">
+      <c r="I28" s="6"/>
+      <c r="J28" s="6">
         <v>1.3</v>
       </c>
-      <c r="J28" s="6">
+      <c r="K28" s="6">
         <v>1.4</v>
       </c>
-      <c r="K28" s="6">
+      <c r="L28" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -1816,19 +1907,22 @@
       <c r="E29" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="G29" s="6"/>
+      <c r="F29" s="4">
+        <v>0</v>
+      </c>
       <c r="H29" s="6"/>
-      <c r="I29" s="6">
-        <v>1.3</v>
-      </c>
+      <c r="I29" s="6"/>
       <c r="J29" s="6">
         <v>1.3</v>
       </c>
       <c r="K29" s="6">
         <v>1.3</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L29" s="6">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -1844,19 +1938,22 @@
       <c r="E30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="G30" s="6"/>
+      <c r="F30" s="4">
+        <v>0</v>
+      </c>
       <c r="H30" s="6"/>
-      <c r="I30" s="6">
+      <c r="I30" s="6"/>
+      <c r="J30" s="6">
         <v>1</v>
       </c>
-      <c r="J30" s="6">
+      <c r="K30" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K30" s="6">
+      <c r="L30" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -1872,19 +1969,22 @@
       <c r="E31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="G31" s="6"/>
+      <c r="F31" s="4">
+        <v>0</v>
+      </c>
       <c r="H31" s="6"/>
-      <c r="I31" s="6">
+      <c r="I31" s="6"/>
+      <c r="J31" s="6">
         <v>1.2</v>
       </c>
-      <c r="J31" s="6">
+      <c r="K31" s="6">
         <v>1.25</v>
       </c>
-      <c r="K31" s="6">
+      <c r="L31" s="6">
         <v>1.3</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -1900,19 +2000,22 @@
       <c r="E32" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G32" s="6"/>
+      <c r="F32" s="4">
+        <v>0</v>
+      </c>
       <c r="H32" s="6"/>
-      <c r="I32" s="6">
+      <c r="I32" s="6"/>
+      <c r="J32" s="6">
         <v>1.4</v>
       </c>
-      <c r="J32" s="6">
+      <c r="K32" s="6">
         <v>1.45</v>
       </c>
-      <c r="K32" s="6">
+      <c r="L32" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -1928,19 +2031,22 @@
       <c r="E33" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="G33" s="6"/>
+      <c r="F33" s="4">
+        <v>0</v>
+      </c>
       <c r="H33" s="6"/>
-      <c r="I33" s="6">
+      <c r="I33" s="6"/>
+      <c r="J33" s="6">
         <v>1</v>
       </c>
-      <c r="J33" s="6">
+      <c r="K33" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K33" s="6">
+      <c r="L33" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -1956,19 +2062,22 @@
       <c r="E34" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G34" s="6"/>
+      <c r="F34" s="4">
+        <v>0</v>
+      </c>
       <c r="H34" s="6"/>
-      <c r="I34" s="6">
+      <c r="I34" s="6"/>
+      <c r="J34" s="6">
         <v>1.05</v>
       </c>
-      <c r="J34" s="6">
+      <c r="K34" s="6">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K34" s="6">
+      <c r="L34" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -1984,19 +2093,22 @@
       <c r="E35" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="G35" s="6"/>
+      <c r="F35" s="4">
+        <v>0</v>
+      </c>
       <c r="H35" s="6"/>
-      <c r="I35" s="6">
+      <c r="I35" s="6"/>
+      <c r="J35" s="6">
         <v>0.9</v>
       </c>
-      <c r="J35" s="6">
+      <c r="K35" s="6">
         <v>1</v>
       </c>
-      <c r="K35" s="6">
+      <c r="L35" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -2012,19 +2124,22 @@
       <c r="E36" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="G36" s="6"/>
+      <c r="F36" s="4">
+        <v>0</v>
+      </c>
       <c r="H36" s="6"/>
-      <c r="I36" s="6">
-        <v>1.5</v>
-      </c>
+      <c r="I36" s="6"/>
       <c r="J36" s="6">
         <v>1.5</v>
       </c>
       <c r="K36" s="6">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36" s="6">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -2040,19 +2155,22 @@
       <c r="E37" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G37" s="6"/>
+      <c r="F37" s="4">
+        <v>0</v>
+      </c>
       <c r="H37" s="6"/>
-      <c r="I37" s="6">
+      <c r="I37" s="6"/>
+      <c r="J37" s="6">
         <v>1</v>
       </c>
-      <c r="J37" s="6">
+      <c r="K37" s="6">
         <v>1.05</v>
       </c>
-      <c r="K37" s="6">
+      <c r="L37" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -2068,19 +2186,22 @@
       <c r="E38" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G38" s="6"/>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
       <c r="H38" s="6"/>
-      <c r="I38" s="6">
+      <c r="I38" s="6"/>
+      <c r="J38" s="6">
         <v>0.8</v>
       </c>
-      <c r="J38" s="6">
+      <c r="K38" s="6">
         <v>0.9</v>
       </c>
-      <c r="K38" s="6">
+      <c r="L38" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -2096,19 +2217,22 @@
       <c r="E39" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="G39" s="6"/>
+      <c r="F39" s="4">
+        <v>0</v>
+      </c>
       <c r="H39" s="6"/>
-      <c r="I39" s="6">
+      <c r="I39" s="6"/>
+      <c r="J39" s="6">
         <v>0.6</v>
       </c>
-      <c r="J39" s="6">
+      <c r="K39" s="6">
         <v>0.8</v>
       </c>
-      <c r="K39" s="6">
+      <c r="L39" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -2124,19 +2248,22 @@
       <c r="E40" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="G40" s="6"/>
+      <c r="F40" s="4">
+        <v>0</v>
+      </c>
       <c r="H40" s="6"/>
-      <c r="I40" s="6">
+      <c r="I40" s="6"/>
+      <c r="J40" s="6">
         <v>0.9</v>
       </c>
-      <c r="J40" s="6">
+      <c r="K40" s="6">
         <v>0.95</v>
       </c>
-      <c r="K40" s="6">
+      <c r="L40" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -2152,19 +2279,22 @@
       <c r="E41" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G41" s="6"/>
+      <c r="F41" s="4">
+        <v>0</v>
+      </c>
       <c r="H41" s="6"/>
-      <c r="I41" s="6">
-        <v>1</v>
-      </c>
+      <c r="I41" s="6"/>
       <c r="J41" s="6">
         <v>1</v>
       </c>
       <c r="K41" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L41" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -2180,19 +2310,22 @@
       <c r="E42" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="G42" s="6"/>
+      <c r="F42" s="4">
+        <v>0</v>
+      </c>
       <c r="H42" s="6"/>
-      <c r="I42" s="6">
+      <c r="I42" s="6"/>
+      <c r="J42" s="6">
         <v>0.1</v>
       </c>
-      <c r="J42" s="6">
+      <c r="K42" s="6">
         <v>0.15</v>
       </c>
-      <c r="K42" s="6">
+      <c r="L42" s="6">
         <v>0.2</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -2208,19 +2341,22 @@
       <c r="E43" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="G43" s="6"/>
+      <c r="F43" s="4">
+        <v>0</v>
+      </c>
       <c r="H43" s="6"/>
-      <c r="I43" s="6">
+      <c r="I43" s="6"/>
+      <c r="J43" s="6">
         <v>0.5</v>
       </c>
-      <c r="J43" s="6">
+      <c r="K43" s="6">
         <v>0.6</v>
       </c>
-      <c r="K43" s="6">
+      <c r="L43" s="6">
         <v>0.8</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -2236,19 +2372,22 @@
       <c r="E44" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G44" s="6"/>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
       <c r="H44" s="6"/>
-      <c r="I44" s="6">
+      <c r="I44" s="6"/>
+      <c r="J44" s="6">
         <v>0.2</v>
       </c>
-      <c r="J44" s="6">
+      <c r="K44" s="6">
         <v>0.25</v>
       </c>
-      <c r="K44" s="6">
+      <c r="L44" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -2264,19 +2403,22 @@
       <c r="E45" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="G45" s="6"/>
+      <c r="F45" s="4">
+        <v>0</v>
+      </c>
       <c r="H45" s="6"/>
-      <c r="I45" s="6">
+      <c r="I45" s="6"/>
+      <c r="J45" s="6">
         <v>1.4</v>
       </c>
-      <c r="J45" s="6">
+      <c r="K45" s="6">
         <v>1.45</v>
       </c>
-      <c r="K45" s="6">
+      <c r="L45" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -2292,19 +2434,22 @@
       <c r="E46" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G46" s="6"/>
+      <c r="F46" s="4">
+        <v>0</v>
+      </c>
       <c r="H46" s="6"/>
-      <c r="I46" s="6">
+      <c r="I46" s="6"/>
+      <c r="J46" s="6">
         <v>0.2</v>
       </c>
-      <c r="J46" s="6">
+      <c r="K46" s="6">
         <v>0.3</v>
       </c>
-      <c r="K46" s="6">
+      <c r="L46" s="6">
         <v>0.4</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2320,19 +2465,22 @@
       <c r="E47" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="G47" s="6"/>
+      <c r="F47" s="4">
+        <v>0</v>
+      </c>
       <c r="H47" s="6"/>
-      <c r="I47" s="6">
+      <c r="I47" s="6"/>
+      <c r="J47" s="6">
         <v>0.15</v>
       </c>
-      <c r="J47" s="6">
+      <c r="K47" s="6">
         <v>0.2</v>
       </c>
-      <c r="K47" s="6">
+      <c r="L47" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -2348,15 +2496,18 @@
       <c r="E48" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="G48" s="6"/>
+      <c r="F48" s="4">
+        <v>0</v>
+      </c>
       <c r="H48" s="6"/>
-      <c r="I48" s="6">
+      <c r="I48" s="6"/>
+      <c r="J48" s="6">
         <v>1.2</v>
       </c>
-      <c r="J48" s="6">
+      <c r="K48" s="6">
         <v>1.3</v>
       </c>
-      <c r="K48" s="6">
+      <c r="L48" s="6">
         <v>1.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[DEV]: Column is_billed_per_case deleted
</commit_message>
<xml_diff>
--- a/data_folder/mapping/mapping_product.xlsx
+++ b/data_folder/mapping/mapping_product.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\workshop\RevAcc\data_folder\mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D35256-91CB-4186-A958-BB94AFB6EAD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A930BFC-0D28-467C-9A2E-35F646330E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="175">
   <si>
     <t>Amora</t>
   </si>
@@ -562,9 +562,6 @@
   </si>
   <si>
     <t>palier_knorr_superior-40000_uvc</t>
-  </si>
-  <si>
-    <t>is_billed_per_case</t>
   </si>
 </sst>
 </file>
@@ -639,10 +636,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="13">
     <dxf>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -696,21 +690,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:L48" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:L48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{D6F1DC80-59FF-426F-9473-675A434B4902}" name="is_billed_per_case" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{5275C952-1BE3-4F8C-914D-044138271CA5}" name="palier_knorr_25000-35000_uvc" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{DEC7AB06-4B54-4173-A4F4-A7451A605C99}" name="palier_knorr_35000-40000_uvc" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{A2C17C36-21F5-4862-AD48-4801B244CECB}" name="palier_knorr_superior-40000_uvc" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}" name="Tableau1" displayName="Tableau1" ref="A1:K48" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K48" xr:uid="{4881BBFE-6E41-44C4-8CFE-1343CC13A1A1}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{F13D4C14-C6D9-4CA4-94EC-E5E38C315D54}" name="brand" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{A1B48B44-CAF8-4F6A-8E0D-3D34DDDB098A}" name="categories" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{B48CA807-13B1-42AC-A3A6-F1B85D613046}" name="keywords_brands" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{89F5A264-D9A1-4704-9B71-FE0DC8313D37}" name="keywords_others" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{DADD4353-00F4-4AAA-9075-8166CE756080}" name="product_name" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{672F9D49-6FE1-4A9E-ACA9-F7CAB1864A3A}" name="palier_dressing+maizena+TVB_25000-35000_uvc" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{2E74C8C6-542F-4CC8-8C88-C724B631E1A3}" name="palier_dressing+maizena+TVB_35000-40000_uvc" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{0049599E-E785-434A-92AE-F8F0EBECF4A7}" name="palier_dressing+maizena+TVB_superior-40000_uvc" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{5275C952-1BE3-4F8C-914D-044138271CA5}" name="palier_knorr_25000-35000_uvc" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{DEC7AB06-4B54-4173-A4F4-A7451A605C99}" name="palier_knorr_35000-40000_uvc" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{A2C17C36-21F5-4862-AD48-4801B244CECB}" name="palier_knorr_superior-40000_uvc" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -979,22 +972,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="53.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="46.42578125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="51" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="49.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="52.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="5" width="48.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="48.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="32.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>56</v>
       </c>
@@ -1011,28 +1004,25 @@
         <v>53</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="L1" s="2" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1048,23 +1038,20 @@
       <c r="E2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="4">
-        <v>1</v>
+      <c r="F2" s="6">
+        <v>0.2</v>
       </c>
       <c r="G2" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I2" s="6">
         <v>0.5</v>
       </c>
+      <c r="I2" s="6"/>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1080,23 +1067,20 @@
       <c r="E3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F3" s="4">
-        <v>0</v>
+      <c r="F3" s="6">
+        <v>0.3</v>
       </c>
       <c r="G3" s="6">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H3" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="I3" s="6">
         <v>0.6</v>
       </c>
+      <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1112,23 +1096,20 @@
       <c r="E4" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="4">
-        <v>0</v>
+      <c r="F4" s="6">
+        <v>1.2</v>
       </c>
       <c r="G4" s="6">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="H4" s="6">
-        <v>1.3</v>
-      </c>
-      <c r="I4" s="6">
         <v>1.5</v>
       </c>
+      <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1144,23 +1125,20 @@
       <c r="E5" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="4">
-        <v>0</v>
+      <c r="F5" s="6">
+        <v>0.6</v>
       </c>
       <c r="G5" s="6">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="H5" s="6">
-        <v>0.7</v>
-      </c>
-      <c r="I5" s="6">
         <v>0.9</v>
       </c>
+      <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1176,23 +1154,20 @@
       <c r="E6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="4">
-        <v>0</v>
+      <c r="F6" s="6">
+        <v>0.2</v>
       </c>
       <c r="G6" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H6" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I6" s="6">
         <v>0.5</v>
       </c>
+      <c r="I6" s="6"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -1208,23 +1183,20 @@
       <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="4">
-        <v>0</v>
+      <c r="F7" s="6">
+        <v>0.1</v>
       </c>
       <c r="G7" s="6">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H7" s="6">
-        <v>0.15</v>
-      </c>
-      <c r="I7" s="6">
         <v>0.2</v>
       </c>
+      <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1240,23 +1212,20 @@
       <c r="E8" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="4">
-        <v>0</v>
+      <c r="F8" s="6">
+        <v>0.3</v>
       </c>
       <c r="G8" s="6">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="I8" s="6">
         <v>0.6</v>
       </c>
+      <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1272,23 +1241,20 @@
       <c r="E9" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="4">
-        <v>0</v>
+      <c r="F9" s="6">
+        <v>0.2</v>
       </c>
       <c r="G9" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H9" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I9" s="6">
         <v>0.4</v>
       </c>
+      <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1304,23 +1270,20 @@
       <c r="E10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="4">
-        <v>0</v>
+      <c r="F10" s="6">
+        <v>0.3</v>
       </c>
       <c r="G10" s="6">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H10" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="I10" s="6">
         <v>0.6</v>
       </c>
+      <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1336,23 +1299,20 @@
       <c r="E11" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="F11" s="4">
-        <v>0</v>
+      <c r="F11" s="6">
+        <v>0.1</v>
       </c>
       <c r="G11" s="6">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H11" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="I11" s="6">
         <v>0.3</v>
       </c>
+      <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -1368,23 +1328,20 @@
       <c r="E12" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F12" s="4">
-        <v>0</v>
+      <c r="F12" s="6">
+        <v>0.1</v>
       </c>
       <c r="G12" s="6">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="H12" s="6">
-        <v>0.12</v>
-      </c>
-      <c r="I12" s="6">
         <v>0.15</v>
       </c>
+      <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1400,23 +1357,20 @@
       <c r="E13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="F13" s="4">
-        <v>0</v>
+      <c r="F13" s="6">
+        <v>0.4</v>
       </c>
       <c r="G13" s="6">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="H13" s="6">
-        <v>0.45</v>
-      </c>
-      <c r="I13" s="6">
         <v>0.5</v>
       </c>
+      <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
@@ -1432,23 +1386,20 @@
       <c r="E14" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="4">
-        <v>0</v>
+      <c r="F14" s="6">
+        <v>0.3</v>
       </c>
       <c r="G14" s="6">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="H14" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="I14" s="6">
         <v>0.45</v>
       </c>
+      <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -1464,23 +1415,20 @@
       <c r="E15" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="4">
-        <v>0</v>
+      <c r="F15" s="6">
+        <v>0.05</v>
       </c>
       <c r="G15" s="6">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="H15" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="I15" s="6">
         <v>0.15</v>
       </c>
+      <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1496,23 +1444,20 @@
       <c r="E16" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="4">
-        <v>0</v>
+      <c r="F16" s="6">
+        <v>1</v>
       </c>
       <c r="G16" s="6">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H16" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="I16" s="6">
         <v>1.1499999999999999</v>
       </c>
+      <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1528,23 +1473,20 @@
       <c r="E17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="4">
-        <v>0</v>
+      <c r="F17" s="6">
+        <v>0.2</v>
       </c>
       <c r="G17" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H17" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I17" s="6">
         <v>0.5</v>
       </c>
+      <c r="I17" s="6"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>4</v>
       </c>
@@ -1560,23 +1502,20 @@
       <c r="E18" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="4">
-        <v>0</v>
+      <c r="F18" s="6">
+        <v>1</v>
       </c>
       <c r="G18" s="6">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="H18" s="6">
-        <v>1.05</v>
-      </c>
-      <c r="I18" s="6">
         <v>1.1000000000000001</v>
       </c>
+      <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>4</v>
       </c>
@@ -1592,23 +1531,20 @@
       <c r="E19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="4">
-        <v>0</v>
+      <c r="F19" s="6">
+        <v>0.2</v>
       </c>
       <c r="G19" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="H19" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="I19" s="6">
         <v>0.4</v>
       </c>
+      <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>4</v>
       </c>
@@ -1624,23 +1560,20 @@
       <c r="E20" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F20" s="4">
-        <v>0</v>
+      <c r="F20" s="6">
+        <v>0.5</v>
       </c>
       <c r="G20" s="6">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="H20" s="6">
-        <v>0.6</v>
-      </c>
-      <c r="I20" s="6">
         <v>0.8</v>
       </c>
+      <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1656,23 +1589,20 @@
       <c r="E21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F21" s="4">
-        <v>0</v>
+      <c r="F21" s="6">
+        <v>0.3</v>
       </c>
       <c r="G21" s="6">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="H21" s="6">
-        <v>0.35</v>
-      </c>
-      <c r="I21" s="6">
         <v>0.45</v>
       </c>
+      <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>5</v>
       </c>
@@ -1688,8 +1618,8 @@
       <c r="E22" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F22" s="4">
-        <v>0</v>
+      <c r="F22" s="6">
+        <v>2.2000000000000002</v>
       </c>
       <c r="G22" s="6">
         <v>2.2000000000000002</v>
@@ -1697,14 +1627,11 @@
       <c r="H22" s="6">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I22" s="6">
-        <v>2.2000000000000002</v>
-      </c>
+      <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1720,23 +1647,20 @@
       <c r="E23" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="4">
-        <v>0</v>
+      <c r="F23" s="6">
+        <v>1.2</v>
       </c>
       <c r="G23" s="6">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="H23" s="6">
-        <v>1.25</v>
-      </c>
-      <c r="I23" s="6">
         <v>1.3</v>
       </c>
+      <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -1752,22 +1676,19 @@
       <c r="E24" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F24" s="4">
-        <v>0</v>
-      </c>
+      <c r="G24" s="6"/>
       <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
+      <c r="I24" s="6">
+        <v>1.2</v>
+      </c>
       <c r="J24" s="6">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K24" s="6">
-        <v>1.3</v>
-      </c>
-      <c r="L24" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -1783,22 +1704,19 @@
       <c r="E25" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F25" s="4">
-        <v>0</v>
-      </c>
+      <c r="G25" s="6"/>
       <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
+      <c r="I25" s="6">
+        <v>1</v>
+      </c>
       <c r="J25" s="6">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K25" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L25" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -1814,22 +1732,19 @@
       <c r="E26" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F26" s="4">
-        <v>0</v>
-      </c>
+      <c r="G26" s="6"/>
       <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
+      <c r="I26" s="6">
+        <v>1.1000000000000001</v>
+      </c>
       <c r="J26" s="6">
-        <v>1.1000000000000001</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="K26" s="6">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="L26" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -1845,22 +1760,19 @@
       <c r="E27" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F27" s="4">
-        <v>0</v>
-      </c>
+      <c r="G27" s="6"/>
       <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
+      <c r="I27" s="6">
+        <v>1.3</v>
+      </c>
       <c r="J27" s="6">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="K27" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="L27" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -1876,22 +1788,19 @@
       <c r="E28" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F28" s="4">
-        <v>0</v>
-      </c>
+      <c r="G28" s="6"/>
       <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
+      <c r="I28" s="6">
+        <v>1.3</v>
+      </c>
       <c r="J28" s="6">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="K28" s="6">
-        <v>1.4</v>
-      </c>
-      <c r="L28" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -1907,22 +1816,19 @@
       <c r="E29" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="F29" s="4">
-        <v>0</v>
-      </c>
+      <c r="G29" s="6"/>
       <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
+      <c r="I29" s="6">
+        <v>1.3</v>
+      </c>
       <c r="J29" s="6">
         <v>1.3</v>
       </c>
       <c r="K29" s="6">
         <v>1.3</v>
       </c>
-      <c r="L29" s="6">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -1938,22 +1844,19 @@
       <c r="E30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="4">
-        <v>0</v>
-      </c>
+      <c r="G30" s="6"/>
       <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
+      <c r="I30" s="6">
+        <v>1</v>
+      </c>
       <c r="J30" s="6">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K30" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L30" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -1969,22 +1872,19 @@
       <c r="E31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F31" s="4">
-        <v>0</v>
-      </c>
+      <c r="G31" s="6"/>
       <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
+      <c r="I31" s="6">
+        <v>1.2</v>
+      </c>
       <c r="J31" s="6">
-        <v>1.2</v>
+        <v>1.25</v>
       </c>
       <c r="K31" s="6">
-        <v>1.25</v>
-      </c>
-      <c r="L31" s="6">
         <v>1.3</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -2000,22 +1900,19 @@
       <c r="E32" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F32" s="4">
-        <v>0</v>
-      </c>
+      <c r="G32" s="6"/>
       <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
+      <c r="I32" s="6">
+        <v>1.4</v>
+      </c>
       <c r="J32" s="6">
-        <v>1.4</v>
+        <v>1.45</v>
       </c>
       <c r="K32" s="6">
-        <v>1.45</v>
-      </c>
-      <c r="L32" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -2031,22 +1928,19 @@
       <c r="E33" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F33" s="4">
-        <v>0</v>
-      </c>
+      <c r="G33" s="6"/>
       <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
+      <c r="I33" s="6">
+        <v>1</v>
+      </c>
       <c r="J33" s="6">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K33" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L33" s="6">
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -2062,22 +1956,19 @@
       <c r="E34" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F34" s="4">
-        <v>0</v>
-      </c>
+      <c r="G34" s="6"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
+      <c r="I34" s="6">
+        <v>1.05</v>
+      </c>
       <c r="J34" s="6">
-        <v>1.05</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K34" s="6">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L34" s="6">
         <v>1.2</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -2093,22 +1984,19 @@
       <c r="E35" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="F35" s="4">
-        <v>0</v>
-      </c>
+      <c r="G35" s="6"/>
       <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
+      <c r="I35" s="6">
+        <v>0.9</v>
+      </c>
       <c r="J35" s="6">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K35" s="6">
-        <v>1</v>
-      </c>
-      <c r="L35" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>6</v>
       </c>
@@ -2124,22 +2012,19 @@
       <c r="E36" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F36" s="4">
-        <v>0</v>
-      </c>
+      <c r="G36" s="6"/>
       <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
+      <c r="I36" s="6">
+        <v>1.5</v>
+      </c>
       <c r="J36" s="6">
         <v>1.5</v>
       </c>
       <c r="K36" s="6">
         <v>1.5</v>
       </c>
-      <c r="L36" s="6">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>6</v>
       </c>
@@ -2155,22 +2040,19 @@
       <c r="E37" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F37" s="4">
-        <v>0</v>
-      </c>
+      <c r="G37" s="6"/>
       <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
+      <c r="I37" s="6">
+        <v>1</v>
+      </c>
       <c r="J37" s="6">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="K37" s="6">
-        <v>1.05</v>
-      </c>
-      <c r="L37" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>6</v>
       </c>
@@ -2186,22 +2068,19 @@
       <c r="E38" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F38" s="4">
-        <v>0</v>
-      </c>
+      <c r="G38" s="6"/>
       <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
+      <c r="I38" s="6">
+        <v>0.8</v>
+      </c>
       <c r="J38" s="6">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K38" s="6">
-        <v>0.9</v>
-      </c>
-      <c r="L38" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>6</v>
       </c>
@@ -2217,22 +2096,19 @@
       <c r="E39" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F39" s="4">
-        <v>0</v>
-      </c>
+      <c r="G39" s="6"/>
       <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
+      <c r="I39" s="6">
+        <v>0.6</v>
+      </c>
       <c r="J39" s="6">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K39" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="L39" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>6</v>
       </c>
@@ -2248,22 +2124,19 @@
       <c r="E40" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F40" s="4">
-        <v>0</v>
-      </c>
+      <c r="G40" s="6"/>
       <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
+      <c r="I40" s="6">
+        <v>0.9</v>
+      </c>
       <c r="J40" s="6">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="K40" s="6">
-        <v>0.95</v>
-      </c>
-      <c r="L40" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>6</v>
       </c>
@@ -2279,22 +2152,19 @@
       <c r="E41" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F41" s="4">
-        <v>0</v>
-      </c>
+      <c r="G41" s="6"/>
       <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
+      <c r="I41" s="6">
+        <v>1</v>
+      </c>
       <c r="J41" s="6">
         <v>1</v>
       </c>
       <c r="K41" s="6">
         <v>1</v>
       </c>
-      <c r="L41" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>6</v>
       </c>
@@ -2310,22 +2180,19 @@
       <c r="E42" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="F42" s="4">
-        <v>0</v>
-      </c>
+      <c r="G42" s="6"/>
       <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
+      <c r="I42" s="6">
+        <v>0.1</v>
+      </c>
       <c r="J42" s="6">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="K42" s="6">
-        <v>0.15</v>
-      </c>
-      <c r="L42" s="6">
         <v>0.2</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>6</v>
       </c>
@@ -2341,22 +2208,19 @@
       <c r="E43" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F43" s="4">
-        <v>0</v>
-      </c>
+      <c r="G43" s="6"/>
       <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
+      <c r="I43" s="6">
+        <v>0.5</v>
+      </c>
       <c r="J43" s="6">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K43" s="6">
-        <v>0.6</v>
-      </c>
-      <c r="L43" s="6">
         <v>0.8</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>6</v>
       </c>
@@ -2372,22 +2236,19 @@
       <c r="E44" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="F44" s="4">
-        <v>0</v>
-      </c>
+      <c r="G44" s="6"/>
       <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
+      <c r="I44" s="6">
+        <v>0.2</v>
+      </c>
       <c r="J44" s="6">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="K44" s="6">
-        <v>0.25</v>
-      </c>
-      <c r="L44" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>6</v>
       </c>
@@ -2403,22 +2264,19 @@
       <c r="E45" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="4">
-        <v>0</v>
-      </c>
+      <c r="G45" s="6"/>
       <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
+      <c r="I45" s="6">
+        <v>1.4</v>
+      </c>
       <c r="J45" s="6">
-        <v>1.4</v>
+        <v>1.45</v>
       </c>
       <c r="K45" s="6">
-        <v>1.45</v>
-      </c>
-      <c r="L45" s="6">
         <v>1.5</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -2434,22 +2292,19 @@
       <c r="E46" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="F46" s="4">
-        <v>0</v>
-      </c>
+      <c r="G46" s="6"/>
       <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
+      <c r="I46" s="6">
+        <v>0.2</v>
+      </c>
       <c r="J46" s="6">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K46" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="L46" s="6">
         <v>0.4</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2465,22 +2320,19 @@
       <c r="E47" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F47" s="4">
-        <v>0</v>
-      </c>
+      <c r="G47" s="6"/>
       <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
+      <c r="I47" s="6">
+        <v>0.15</v>
+      </c>
       <c r="J47" s="6">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="K47" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="L47" s="6">
         <v>0.3</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>6</v>
       </c>
@@ -2496,18 +2348,15 @@
       <c r="E48" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="F48" s="4">
-        <v>0</v>
-      </c>
+      <c r="G48" s="6"/>
       <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
+      <c r="I48" s="6">
+        <v>1.2</v>
+      </c>
       <c r="J48" s="6">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K48" s="6">
-        <v>1.3</v>
-      </c>
-      <c r="L48" s="6">
         <v>1.4</v>
       </c>
     </row>

</xml_diff>